<commit_message>
data/creation dataset clients et modification dataset ventes_brutes.csv
</commit_message>
<xml_diff>
--- a/data/raw/ventes_brutes.csv.xlsx
+++ b/data/raw/ventes_brutes.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\powerbi-ai-journey\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{90D17C4B-0B85-434D-ACA6-AF1D08BF7575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F31215A-8A3D-44E8-9BCB-11BCC87AAFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1331542A-48BC-4F99-AB05-851732DEAC4F}"/>
   </bookViews>
@@ -179,11 +179,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -191,10 +190,10 @@
   </cellStyles>
   <dxfs count="2">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -213,8 +212,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D8BF3035-7D1A-47F6-80B1-05B121BCABD3}" name="Tableau1" displayName="Tableau1" ref="A1:H13" totalsRowShown="0">
   <autoFilter ref="A1:H13" xr:uid="{D8BF3035-7D1A-47F6-80B1-05B121BCABD3}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{745AD39B-A749-4B0D-951C-40850B7B0C3F}" name="ID_VENTE" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{1384BDF0-6DC2-4AEB-A306-43E87D3C34F0}" name="DATE_VENTE" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{745AD39B-A749-4B0D-951C-40850B7B0C3F}" name="ID_VENTE" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{1384BDF0-6DC2-4AEB-A306-43E87D3C34F0}" name="DATE_VENTE" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{1332752E-6485-44F7-872D-0B2F1CB92983}" name="EMAIL_CLIENT"/>
     <tableColumn id="4" xr3:uid="{B3B54E2D-6120-4E5A-9720-FA5A15B24274}" name="PRODUIT"/>
     <tableColumn id="5" xr3:uid="{ED86EACB-E889-4ED0-B100-8C8935C41948}" name="CATEGORIE"/>
@@ -578,7 +577,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="1">
@@ -604,7 +603,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="1">
@@ -630,7 +629,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="1">
@@ -656,7 +655,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="1">
@@ -679,7 +678,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
+      <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" s="1">
@@ -702,7 +701,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="1">
@@ -728,7 +727,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
+      <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" s="1">
@@ -754,7 +753,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
+      <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" s="1">
@@ -780,7 +779,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="3">
+      <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" s="1">
@@ -806,7 +805,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
+      <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" s="1">
@@ -829,7 +828,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
+      <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" s="1">
@@ -855,7 +854,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="3">
+      <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" s="1">

</xml_diff>